<commit_message>
Regenerate all recode and rename reports
</commit_message>
<xml_diff>
--- a/Resources/Crosswalks/all_recode_variables.xlsx
+++ b/Resources/Crosswalks/all_recode_variables.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H431"/>
+  <dimension ref="A1:H432"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -12994,27 +12994,22 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>tobacco</t>
+          <t>pregnancy</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
           <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G360" t="inlineStr">
-        <is>
-          <t>Not in data dictionary</t>
         </is>
       </c>
       <c r="H360" t="b">
@@ -13024,36 +13019,36 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>hispanic_cuban</t>
+          <t>tobacco</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="D361" t="inlineStr">
-        <is>
-          <t>Hispanic</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>U</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>Not in data dictionary</t>
         </is>
       </c>
       <c r="H361" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="362">
@@ -13064,7 +13059,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>hispanic_mexican</t>
+          <t>hispanic_cuban</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -13099,7 +13094,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>hispanic_other</t>
+          <t>hispanic_mexican</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -13134,7 +13129,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>hispanic_puerto_rican</t>
+          <t>hispanic_other</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -13169,47 +13164,47 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>tobacco</t>
+          <t>hispanic_puerto_rican</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Hispanic</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G365" t="inlineStr">
-        <is>
-          <t>Not in data dictionary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H365" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>disposition</t>
+          <t>tobacco</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
@@ -13244,7 +13239,7 @@
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
@@ -13274,31 +13269,31 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>hispanic_cuban</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="D368" t="inlineStr">
-        <is>
-          <t>Hispanic</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>U</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>Not in data dictionary</t>
         </is>
       </c>
       <c r="H368" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="369">
@@ -13309,7 +13304,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>hispanic_mexican</t>
+          <t>hispanic_cuban</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -13344,7 +13339,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>hispanic_other</t>
+          <t>hispanic_mexican</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -13379,7 +13374,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>hispanic_puerto_rican</t>
+          <t>hispanic_other</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -13414,31 +13409,31 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>injury_acme_place</t>
+          <t>hispanic_puerto_rican</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Hispanic</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>Unspecified Place</t>
-        </is>
-      </c>
-      <c r="G372" t="inlineStr">
-        <is>
-          <t>Not in data dictionary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H372" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="373">
@@ -13454,7 +13449,7 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E373" t="inlineStr">
@@ -13489,7 +13484,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E374" t="inlineStr">
@@ -13524,7 +13519,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E375" t="inlineStr">
@@ -13559,7 +13554,7 @@
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>K</t>
         </is>
       </c>
       <c r="E376" t="inlineStr">
@@ -13594,7 +13589,7 @@
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E377" t="inlineStr">
@@ -13629,7 +13624,7 @@
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E378" t="inlineStr">
@@ -13664,7 +13659,7 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E379" t="inlineStr">
@@ -13694,22 +13689,22 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>tobacco</t>
+          <t>injury_acme_place</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unspecified Place</t>
         </is>
       </c>
       <c r="G380" t="inlineStr">
@@ -13724,17 +13719,17 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>disposition</t>
+          <t>tobacco</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E381" t="inlineStr">
@@ -13769,7 +13764,7 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E382" t="inlineStr">
@@ -13799,31 +13794,31 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>hispanic_cuban</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="D383" t="inlineStr">
-        <is>
-          <t>Hispanic</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>U</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>Not in data dictionary</t>
         </is>
       </c>
       <c r="H383" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="384">
@@ -13834,7 +13829,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>hispanic_mexican</t>
+          <t>hispanic_cuban</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
@@ -13869,7 +13864,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>hispanic_other</t>
+          <t>hispanic_mexican</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
@@ -13904,7 +13899,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>hispanic_puerto_rican</t>
+          <t>hispanic_other</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -13939,31 +13934,31 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>injury_acme_place</t>
+          <t>hispanic_puerto_rican</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Hispanic</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>Unspecified Place</t>
-        </is>
-      </c>
-      <c r="G387" t="inlineStr">
-        <is>
-          <t>Not in data dictionary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H387" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="388">
@@ -13979,7 +13974,7 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
@@ -14014,7 +14009,7 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E389" t="inlineStr">
@@ -14049,7 +14044,7 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="E390" t="inlineStr">
@@ -14084,7 +14079,7 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>G</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
@@ -14119,7 +14114,7 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>K</t>
         </is>
       </c>
       <c r="E392" t="inlineStr">
@@ -14154,7 +14149,7 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E393" t="inlineStr">
@@ -14189,7 +14184,7 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E394" t="inlineStr">
@@ -14219,22 +14214,22 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>tobacco</t>
+          <t>injury_acme_place</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unspecified Place</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
@@ -14249,17 +14244,17 @@
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>disposition</t>
+          <t>tobacco</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E396" t="inlineStr">
@@ -14294,7 +14289,7 @@
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E397" t="inlineStr">
@@ -14324,31 +14319,31 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>hispanic_cuban</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="D398" t="inlineStr">
-        <is>
-          <t>Hispanic</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>U</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>Not in data dictionary</t>
         </is>
       </c>
       <c r="H398" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="399">
@@ -14359,7 +14354,7 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>hispanic_mexican</t>
+          <t>hispanic_cuban</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
@@ -14394,7 +14389,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>hispanic_other</t>
+          <t>hispanic_mexican</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -14429,7 +14424,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>hispanic_puerto_rican</t>
+          <t>hispanic_other</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
@@ -14464,31 +14459,31 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>injury_acme_place</t>
+          <t>hispanic_puerto_rican</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Hispanic</t>
         </is>
       </c>
       <c r="E402" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t>Unspecified Place</t>
-        </is>
-      </c>
-      <c r="G402" t="inlineStr">
-        <is>
-          <t>Not in data dictionary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H402" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="403">
@@ -14504,7 +14499,7 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E403" t="inlineStr">
@@ -14539,7 +14534,7 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E404" t="inlineStr">
@@ -14574,7 +14569,7 @@
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E405" t="inlineStr">
@@ -14609,7 +14604,7 @@
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E406" t="inlineStr">
@@ -14644,7 +14639,7 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>H</t>
         </is>
       </c>
       <c r="E407" t="inlineStr">
@@ -14679,7 +14674,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>K</t>
         </is>
       </c>
       <c r="E408" t="inlineStr">
@@ -14714,7 +14709,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E409" t="inlineStr">
@@ -14749,7 +14744,7 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E410" t="inlineStr">
@@ -14784,7 +14779,7 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>O</t>
         </is>
       </c>
       <c r="E411" t="inlineStr">
@@ -14819,7 +14814,7 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E412" t="inlineStr">
@@ -14849,22 +14844,22 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>tobacco</t>
+          <t>injury_acme_place</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unspecified Place</t>
         </is>
       </c>
       <c r="G413" t="inlineStr">
@@ -14879,17 +14874,17 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>disposition</t>
+          <t>tobacco</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E414" t="inlineStr">
@@ -14924,7 +14919,7 @@
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E415" t="inlineStr">
@@ -14954,31 +14949,31 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>hispanic_cuban</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="D416" t="inlineStr">
-        <is>
-          <t>Hispanic</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>U</t>
         </is>
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>Not in data dictionary</t>
         </is>
       </c>
       <c r="H416" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="417">
@@ -14989,7 +14984,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>hispanic_mexican</t>
+          <t>hispanic_cuban</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -15024,7 +15019,7 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>hispanic_other</t>
+          <t>hispanic_mexican</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -15059,7 +15054,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>hispanic_puerto_rican</t>
+          <t>hispanic_other</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -15094,31 +15089,31 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>injury_acme_place</t>
+          <t>hispanic_puerto_rican</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Hispanic</t>
         </is>
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t>Unspecified Place</t>
-        </is>
-      </c>
-      <c r="G420" t="inlineStr">
-        <is>
-          <t>Not in data dictionary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H420" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="421">
@@ -15129,7 +15124,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>marital_status</t>
+          <t>injury_acme_place</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -15139,12 +15134,12 @@
       </c>
       <c r="E421" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F421" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unspecified Place</t>
         </is>
       </c>
       <c r="G421" t="inlineStr">
@@ -15159,17 +15154,17 @@
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>disposition</t>
+          <t>marital_status</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E422" t="inlineStr">
@@ -15204,7 +15199,7 @@
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E423" t="inlineStr">
@@ -15234,31 +15229,31 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>hispanic_cuban</t>
+          <t>disposition</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="D424" t="inlineStr">
-        <is>
-          <t>Hispanic</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>U</t>
         </is>
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>Not in data dictionary</t>
         </is>
       </c>
       <c r="H424" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="425">
@@ -15269,7 +15264,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>hispanic_mexican</t>
+          <t>hispanic_cuban</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -15304,7 +15299,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>hispanic_other</t>
+          <t>hispanic_mexican</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -15339,7 +15334,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>hispanic_puerto_rican</t>
+          <t>hispanic_other</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
@@ -15374,31 +15369,31 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>injury_acme_place</t>
+          <t>hispanic_puerto_rican</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Hispanic</t>
         </is>
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t>Unspecified Place</t>
-        </is>
-      </c>
-      <c r="G428" t="inlineStr">
-        <is>
-          <t>Not in data dictionary</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H428" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="429">
@@ -15409,7 +15404,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>marital_status</t>
+          <t>injury_acme_place</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
@@ -15419,12 +15414,12 @@
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Unspecified Place</t>
         </is>
       </c>
       <c r="G429" t="inlineStr">
@@ -15444,17 +15439,17 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>pregnancy</t>
+          <t>marital_status</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E430" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>U</t>
         </is>
       </c>
       <c r="F430" t="inlineStr">
@@ -15484,25 +15479,60 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>Not in data dictionary</t>
+        </is>
+      </c>
+      <c r="H431" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>pregnancy</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E431" t="inlineStr">
+      <c r="E432" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="F431" t="inlineStr">
+      <c r="F432" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="G431" t="inlineStr">
+      <c r="G432" t="inlineStr">
         <is>
           <t>Not in data dictionary</t>
         </is>
       </c>
-      <c r="H431" t="b">
+      <c r="H432" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>